<commit_message>
Update QA test execution and summary report
Update test execution results, product navigation findings, and test summary metrics.
</commit_message>
<xml_diff>
--- a/QA_Testing_ECommerce_Portfolio_Updated.xlsx
+++ b/QA_Testing_ECommerce_Portfolio_Updated.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ACER\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{375B3439-7D84-4073-8B84-38B8330A8488}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{480675E5-034C-40A9-AFC3-83D48E6C5C7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Test_Cases" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="386" uniqueCount="275">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="405" uniqueCount="290">
   <si>
     <t>QA TESTING PROJECT | TEST CASES</t>
   </si>
@@ -816,9 +816,6 @@
     <t>Execution Period</t>
   </si>
   <si>
-    <t>05–13 October 2026 (based on recorded dates)</t>
-  </si>
-  <si>
     <t>Test Environment</t>
   </si>
   <si>
@@ -900,9 +897,6 @@
     <t>CONCLUSION</t>
   </si>
   <si>
-    <t>The recorded login and checkout required-field scenarios behaved as expected during the reported executions. The end-to-end product-to-order workflow was observed to complete successfully, including order confirmation and PDF receipt generation. Additional demo-account observations remain preliminary and should be reproduced and assessed separately. These results apply only to the scenarios documented in this report.</t>
-  </si>
-  <si>
     <t>RECOMMENDED NEXT STEPS</t>
   </si>
   <si>
@@ -913,13 +907,80 @@
   </si>
   <si>
     <t>3. Continue with Jira defect lifecycle practice, followed by basic Postman/REST and MySQL exercises aligned with the POSe.id internship description.</t>
+  </si>
+  <si>
+    <t>TC-PRODUCT-001</t>
+  </si>
+  <si>
+    <t>Verify that selecting a product opens the corresponding product detail page.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">User is logged in using the </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>problem_user</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Carlito"/>
+      </rPr>
+      <t xml:space="preserve"> demo account and is on the Inventory page.</t>
+    </r>
+  </si>
+  <si>
+    <t>Sauce Labs Backpack</t>
+  </si>
+  <si>
+    <t>1. Open the Inventory page                      2. Select Sauce Labs Backpack.             3. Observe the product name and information displayed on the resulting page.</t>
+  </si>
+  <si>
+    <t>The Sauce Labs Backpack detail page is displayed with the corresponding product information.</t>
+  </si>
+  <si>
+    <t>The resulting page displayed Sauce Labs Fleece Jacket instead of Sauce Labs Backpack.</t>
+  </si>
+  <si>
+    <t>Product Detail / Navigation</t>
+  </si>
+  <si>
+    <t>problem_user / Sauce Labs Backpack</t>
+  </si>
+  <si>
+    <t>The Sauce Labs Backpack detail page is displayed with matching product information.</t>
+  </si>
+  <si>
+    <t>Observed with problem_user demo account. Related Jira issue: SCRUM-5. Evidence is attached to the issue.</t>
+  </si>
+  <si>
+    <t>2026-10-14</t>
+  </si>
+  <si>
+    <t>Select Sauce Labs Backpack and verify the corresponding product detail page opens</t>
+  </si>
+  <si>
+    <t>05–14 October 2026 (based on recorded dates)</t>
+  </si>
+  <si>
+    <t>Product Detail / Navigatio</t>
+  </si>
+  <si>
+    <t>Selecting Sauce Labs Backpack displayed Sauce Labs Fleece Jacket when using the problem_user demo account.</t>
+  </si>
+  <si>
+    <t>The recorded login scenarios, checkout required-field validation scenarios, and end-to-end product-to-order workflow behaved as expected during the documented executions. One product navigation test case failed when using the problem_user demo account: selecting Sauce Labs Backpack displayed Sauce Labs Fleece Jacket instead. Other exploratory observations remain preliminary and require further verification before being classified as confirmed defects. These results are limited to the documented test scenarios and do not establish the overall quality or production readiness of the application.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="13">
+  <fonts count="15">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -991,6 +1052,14 @@
     <font>
       <sz val="10"/>
       <color rgb="FF243B53"/>
+      <name val="Carlito"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial Unicode MS"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Carlito"/>
     </font>
   </fonts>
@@ -1089,7 +1158,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1112,15 +1181,27 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1133,8 +1214,47 @@
     <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -1142,56 +1262,17 @@
     <xf numFmtId="0" fontId="7" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1405,11 +1486,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H18"/>
   <sheetFormatPr defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
-    <col min="2" max="2" width="16" customWidth="1"/>
+    <col min="2" max="2" width="16.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="14" customWidth="1"/>
     <col min="4" max="5" width="30" customWidth="1"/>
     <col min="6" max="6" width="31" customWidth="1"/>
@@ -1418,40 +1499,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="32" customHeight="1">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
-      <c r="G1" s="8"/>
-      <c r="H1" s="8"/>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
+      <c r="H1" s="13"/>
     </row>
     <row r="2" spans="1:8" ht="30" customHeight="1">
-      <c r="A2" s="9" t="s">
+      <c r="A2" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="9"/>
-      <c r="C2" s="9"/>
-      <c r="D2" s="9"/>
-      <c r="E2" s="9"/>
-      <c r="F2" s="9"/>
-      <c r="G2" s="9"/>
-      <c r="H2" s="9"/>
+      <c r="B2" s="14"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="14"/>
+      <c r="G2" s="14"/>
+      <c r="H2" s="14"/>
     </row>
     <row r="4" spans="1:8" ht="30" customHeight="1">
-      <c r="A4" s="10" t="s">
+      <c r="A4" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="10"/>
-      <c r="C4" s="10"/>
-      <c r="D4" s="10"/>
-      <c r="E4" s="10"/>
-      <c r="F4" s="10"/>
-      <c r="G4" s="10"/>
-      <c r="H4" s="10"/>
+      <c r="B4" s="12"/>
+      <c r="C4" s="12"/>
+      <c r="D4" s="12"/>
+      <c r="E4" s="12"/>
+      <c r="F4" s="12"/>
+      <c r="G4" s="12"/>
+      <c r="H4" s="12"/>
     </row>
     <row r="5" spans="1:8" ht="34" customHeight="1">
       <c r="A5" s="1" t="s">
@@ -1480,227 +1561,227 @@
       </c>
     </row>
     <row r="6" spans="1:8" ht="70" customHeight="1">
-      <c r="A6" s="33" t="s">
+      <c r="A6" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="B6" s="33" t="s">
+      <c r="B6" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="C6" s="33" t="s">
+      <c r="C6" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="D6" s="33" t="s">
+      <c r="D6" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="E6" s="33" t="s">
+      <c r="E6" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="F6" s="32" t="s">
+      <c r="F6" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="G6" s="32" t="s">
+      <c r="G6" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H6" s="32" t="s">
+      <c r="H6" s="8" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="70" customHeight="1">
-      <c r="A7" s="33" t="s">
+      <c r="A7" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="B7" s="33" t="s">
+      <c r="B7" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="C7" s="33" t="s">
+      <c r="C7" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="D7" s="33" t="s">
+      <c r="D7" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="E7" s="33" t="s">
+      <c r="E7" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="F7" s="32" t="s">
+      <c r="F7" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="G7" s="32" t="s">
+      <c r="G7" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="H7" s="32" t="s">
+      <c r="H7" s="8" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="70" customHeight="1">
-      <c r="A8" s="33" t="s">
+      <c r="A8" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="B8" s="33" t="s">
+      <c r="B8" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="C8" s="33" t="s">
+      <c r="C8" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="D8" s="33" t="s">
+      <c r="D8" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="E8" s="33" t="s">
+      <c r="E8" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="F8" s="32" t="s">
+      <c r="F8" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="G8" s="32" t="s">
+      <c r="G8" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="H8" s="32" t="s">
+      <c r="H8" s="8" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="70" customHeight="1">
-      <c r="A9" s="33" t="s">
+      <c r="A9" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="B9" s="33" t="s">
+      <c r="B9" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="C9" s="33" t="s">
+      <c r="C9" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="D9" s="33" t="s">
+      <c r="D9" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="E9" s="33" t="s">
+      <c r="E9" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="F9" s="32" t="s">
+      <c r="F9" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="G9" s="32" t="s">
+      <c r="G9" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="H9" s="32" t="s">
+      <c r="H9" s="8" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="70" customHeight="1">
-      <c r="A10" s="33" t="s">
+      <c r="A10" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="B10" s="33" t="s">
+      <c r="B10" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="C10" s="33" t="s">
+      <c r="C10" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="D10" s="33" t="s">
+      <c r="D10" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="E10" s="33" t="s">
+      <c r="E10" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="F10" s="32" t="s">
+      <c r="F10" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="G10" s="32" t="s">
+      <c r="G10" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="H10" s="32" t="s">
+      <c r="H10" s="8" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="70" customHeight="1">
-      <c r="A11" s="33" t="s">
+      <c r="A11" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="B11" s="33" t="s">
+      <c r="B11" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="C11" s="33" t="s">
+      <c r="C11" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="D11" s="33" t="s">
+      <c r="D11" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="E11" s="33" t="s">
+      <c r="E11" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="F11" s="32" t="s">
+      <c r="F11" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="G11" s="32" t="s">
+      <c r="G11" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="H11" s="32" t="s">
+      <c r="H11" s="8" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="70" customHeight="1">
-      <c r="A12" s="33" t="s">
+      <c r="A12" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="B12" s="33" t="s">
+      <c r="B12" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="C12" s="33" t="s">
+      <c r="C12" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="D12" s="33" t="s">
+      <c r="D12" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="E12" s="33" t="s">
+      <c r="E12" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="F12" s="32" t="s">
+      <c r="F12" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="G12" s="32" t="s">
+      <c r="G12" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="H12" s="32" t="s">
+      <c r="H12" s="8" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="70" customHeight="1">
-      <c r="A13" s="33" t="s">
+      <c r="A13" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="B13" s="33" t="s">
+      <c r="B13" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="C13" s="33" t="s">
+      <c r="C13" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="D13" s="33" t="s">
+      <c r="D13" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="E13" s="33" t="s">
+      <c r="E13" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="F13" s="32" t="s">
+      <c r="F13" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="G13" s="32" t="s">
+      <c r="G13" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="H13" s="32" t="s">
+      <c r="H13" s="8" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="86" customHeight="1">
-      <c r="A14" s="34" t="s">
+      <c r="A14" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="B14" s="34" t="s">
+      <c r="B14" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="C14" s="34" t="s">
+      <c r="C14" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="D14" s="34" t="s">
+      <c r="D14" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="E14" s="34" t="s">
+      <c r="E14" s="10" t="s">
         <v>63</v>
       </c>
       <c r="F14" s="7" t="s">
@@ -1714,19 +1795,19 @@
       </c>
     </row>
     <row r="15" spans="1:8" ht="86" customHeight="1">
-      <c r="A15" s="34" t="s">
+      <c r="A15" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="B15" s="34" t="s">
+      <c r="B15" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="C15" s="34" t="s">
+      <c r="C15" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="D15" s="34" t="s">
+      <c r="D15" s="10" t="s">
         <v>69</v>
       </c>
-      <c r="E15" s="34" t="s">
+      <c r="E15" s="10" t="s">
         <v>70</v>
       </c>
       <c r="F15" s="7" t="s">
@@ -1740,19 +1821,19 @@
       </c>
     </row>
     <row r="16" spans="1:8" ht="86" customHeight="1">
-      <c r="A16" s="34" t="s">
+      <c r="A16" s="10" t="s">
         <v>74</v>
       </c>
-      <c r="B16" s="34" t="s">
+      <c r="B16" s="10" t="s">
         <v>75</v>
       </c>
-      <c r="C16" s="34" t="s">
+      <c r="C16" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="D16" s="34" t="s">
+      <c r="D16" s="10" t="s">
         <v>76</v>
       </c>
-      <c r="E16" s="34" t="s">
+      <c r="E16" s="10" t="s">
         <v>70</v>
       </c>
       <c r="F16" s="7" t="s">
@@ -1766,19 +1847,19 @@
       </c>
     </row>
     <row r="17" spans="1:8" ht="150" customHeight="1">
-      <c r="A17" s="34" t="s">
+      <c r="A17" s="10" t="s">
         <v>80</v>
       </c>
-      <c r="B17" s="34" t="s">
+      <c r="B17" s="10" t="s">
         <v>81</v>
       </c>
-      <c r="C17" s="34" t="s">
+      <c r="C17" s="10" t="s">
         <v>82</v>
       </c>
-      <c r="D17" s="34" t="s">
+      <c r="D17" s="10" t="s">
         <v>83</v>
       </c>
-      <c r="E17" s="34" t="s">
+      <c r="E17" s="10" t="s">
         <v>84</v>
       </c>
       <c r="F17" s="7" t="s">
@@ -1789,6 +1870,32 @@
       </c>
       <c r="H17" s="7" t="s">
         <v>87</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" ht="70">
+      <c r="A18" s="35" t="s">
+        <v>273</v>
+      </c>
+      <c r="B18" s="35" t="s">
+        <v>273</v>
+      </c>
+      <c r="C18" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="D18" s="7" t="s">
+        <v>274</v>
+      </c>
+      <c r="E18" s="7" t="s">
+        <v>275</v>
+      </c>
+      <c r="F18" s="36" t="s">
+        <v>276</v>
+      </c>
+      <c r="G18" s="5" t="s">
+        <v>277</v>
+      </c>
+      <c r="H18" s="7" t="s">
+        <v>278</v>
       </c>
     </row>
   </sheetData>
@@ -1797,13 +1904,15 @@
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A4:H4"/>
   </mergeCells>
+  <phoneticPr fontId="14" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:I20"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
@@ -1818,89 +1927,89 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="32" customHeight="1">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="13" t="s">
         <v>88</v>
       </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
-      <c r="G1" s="8"/>
-      <c r="H1" s="8"/>
-      <c r="I1" s="8"/>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
+      <c r="H1" s="13"/>
+      <c r="I1" s="13"/>
     </row>
     <row r="2" spans="1:9" ht="30" customHeight="1">
-      <c r="A2" s="9" t="s">
+      <c r="A2" s="14" t="s">
         <v>89</v>
       </c>
-      <c r="B2" s="9"/>
-      <c r="C2" s="9"/>
-      <c r="D2" s="9"/>
-      <c r="E2" s="9"/>
-      <c r="F2" s="9"/>
-      <c r="G2" s="9"/>
-      <c r="H2" s="9"/>
-      <c r="I2" s="9"/>
+      <c r="B2" s="14"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="14"/>
+      <c r="G2" s="14"/>
+      <c r="H2" s="14"/>
+      <c r="I2" s="14"/>
     </row>
     <row r="4" spans="1:9">
-      <c r="A4" s="11" t="s">
+      <c r="A4" s="15" t="s">
         <v>90</v>
       </c>
-      <c r="B4" s="11"/>
-      <c r="C4" s="12" t="s">
+      <c r="B4" s="15"/>
+      <c r="C4" s="16" t="s">
         <v>91</v>
       </c>
-      <c r="D4" s="12"/>
-      <c r="E4" s="13" t="s">
+      <c r="D4" s="16"/>
+      <c r="E4" s="17" t="s">
         <v>92</v>
       </c>
-      <c r="F4" s="13"/>
-      <c r="G4" s="14" t="s">
+      <c r="F4" s="17"/>
+      <c r="G4" s="18" t="s">
         <v>93</v>
       </c>
-      <c r="H4" s="14"/>
+      <c r="H4" s="18"/>
       <c r="I4" s="3" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="28" customHeight="1">
-      <c r="A5" s="15">
-        <f>COUNTA(A9:A20)</f>
+      <c r="A5" s="11">
+        <f>COUNTA(A9:A21)</f>
+        <v>13</v>
+      </c>
+      <c r="B5" s="11"/>
+      <c r="C5" s="11">
+        <f>COUNTIF(F9:F21,"PASS")</f>
         <v>12</v>
       </c>
-      <c r="B5" s="15"/>
-      <c r="C5" s="15">
-        <f>COUNTIF(F9:F20,"PASS")</f>
-        <v>12</v>
-      </c>
-      <c r="D5" s="15"/>
-      <c r="E5" s="15">
-        <f>COUNTIF(F9:F20,"FAIL")</f>
+      <c r="D5" s="11"/>
+      <c r="E5" s="11">
+        <f>COUNTIF(F9:F21,"FAIL")</f>
+        <v>1</v>
+      </c>
+      <c r="F5" s="11"/>
+      <c r="G5" s="11">
+        <f>COUNTIF(F9:F21,"BLOCKED")</f>
         <v>0</v>
       </c>
-      <c r="F5" s="15"/>
-      <c r="G5" s="15">
-        <f>COUNTIF(F9:F20,"BLOCKED")</f>
-        <v>0</v>
-      </c>
-      <c r="H5" s="15"/>
+      <c r="H5" s="11"/>
       <c r="I5" s="4" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="28" customHeight="1">
-      <c r="A7" s="10" t="s">
+      <c r="A7" s="12" t="s">
         <v>96</v>
       </c>
-      <c r="B7" s="10"/>
-      <c r="C7" s="10"/>
-      <c r="D7" s="10"/>
-      <c r="E7" s="10"/>
-      <c r="F7" s="10"/>
-      <c r="G7" s="10"/>
-      <c r="H7" s="10"/>
-      <c r="I7" s="10"/>
+      <c r="B7" s="12"/>
+      <c r="C7" s="12"/>
+      <c r="D7" s="12"/>
+      <c r="E7" s="12"/>
+      <c r="F7" s="12"/>
+      <c r="G7" s="12"/>
+      <c r="H7" s="12"/>
+      <c r="I7" s="12"/>
     </row>
     <row r="8" spans="1:9" ht="34" customHeight="1">
       <c r="A8" s="1" t="s">
@@ -1932,260 +2041,260 @@
       </c>
     </row>
     <row r="9" spans="1:9" ht="62" customHeight="1">
-      <c r="A9" s="33" t="s">
+      <c r="A9" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="B9" s="33" t="s">
+      <c r="B9" s="9" t="s">
         <v>104</v>
       </c>
-      <c r="C9" s="33" t="s">
+      <c r="C9" s="9" t="s">
         <v>105</v>
       </c>
-      <c r="D9" s="33" t="s">
+      <c r="D9" s="9" t="s">
         <v>106</v>
       </c>
-      <c r="E9" s="33" t="s">
+      <c r="E9" s="9" t="s">
         <v>107</v>
       </c>
-      <c r="F9" s="33" t="s">
+      <c r="F9" s="9" t="s">
         <v>91</v>
       </c>
-      <c r="G9" s="33" t="s">
+      <c r="G9" s="9" t="s">
         <v>108</v>
       </c>
-      <c r="H9" s="33" t="s">
+      <c r="H9" s="9" t="s">
         <v>109</v>
       </c>
-      <c r="I9" s="32" t="s">
+      <c r="I9" s="8" t="s">
         <v>110</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="62" customHeight="1">
-      <c r="A10" s="33" t="s">
+      <c r="A10" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="B10" s="33" t="s">
+      <c r="B10" s="9" t="s">
         <v>111</v>
       </c>
-      <c r="C10" s="33" t="s">
+      <c r="C10" s="9" t="s">
         <v>112</v>
       </c>
-      <c r="D10" s="33" t="s">
+      <c r="D10" s="9" t="s">
         <v>113</v>
       </c>
-      <c r="E10" s="33" t="s">
+      <c r="E10" s="9" t="s">
         <v>114</v>
       </c>
-      <c r="F10" s="33" t="s">
+      <c r="F10" s="9" t="s">
         <v>91</v>
       </c>
-      <c r="G10" s="33" t="s">
+      <c r="G10" s="9" t="s">
         <v>115</v>
       </c>
-      <c r="H10" s="33" t="s">
+      <c r="H10" s="9" t="s">
         <v>109</v>
       </c>
-      <c r="I10" s="32" t="s">
+      <c r="I10" s="8" t="s">
         <v>116</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="62" customHeight="1">
-      <c r="A11" s="33" t="s">
+      <c r="A11" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="B11" s="33" t="s">
+      <c r="B11" s="9" t="s">
         <v>117</v>
       </c>
-      <c r="C11" s="33" t="s">
+      <c r="C11" s="9" t="s">
         <v>118</v>
       </c>
-      <c r="D11" s="33" t="s">
+      <c r="D11" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="E11" s="33" t="s">
+      <c r="E11" s="9" t="s">
         <v>119</v>
       </c>
-      <c r="F11" s="33" t="s">
+      <c r="F11" s="9" t="s">
         <v>91</v>
       </c>
-      <c r="G11" s="33" t="s">
+      <c r="G11" s="9" t="s">
         <v>108</v>
       </c>
-      <c r="H11" s="33" t="s">
+      <c r="H11" s="9" t="s">
         <v>109</v>
       </c>
-      <c r="I11" s="32" t="s">
+      <c r="I11" s="8" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="62" customHeight="1">
-      <c r="A12" s="33" t="s">
+      <c r="A12" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="B12" s="33" t="s">
+      <c r="B12" s="9" t="s">
         <v>121</v>
       </c>
-      <c r="C12" s="33" t="s">
+      <c r="C12" s="9" t="s">
         <v>122</v>
       </c>
-      <c r="D12" s="33" t="s">
+      <c r="D12" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="E12" s="33" t="s">
+      <c r="E12" s="9" t="s">
         <v>119</v>
       </c>
-      <c r="F12" s="33" t="s">
+      <c r="F12" s="9" t="s">
         <v>91</v>
       </c>
-      <c r="G12" s="33" t="s">
+      <c r="G12" s="9" t="s">
         <v>108</v>
       </c>
-      <c r="H12" s="33" t="s">
+      <c r="H12" s="9" t="s">
         <v>109</v>
       </c>
-      <c r="I12" s="32" t="s">
+      <c r="I12" s="8" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="62" customHeight="1">
-      <c r="A13" s="33" t="s">
+      <c r="A13" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="B13" s="33" t="s">
+      <c r="B13" s="9" t="s">
         <v>123</v>
       </c>
-      <c r="C13" s="33" t="s">
+      <c r="C13" s="9" t="s">
         <v>124</v>
       </c>
-      <c r="D13" s="33" t="s">
+      <c r="D13" s="9" t="s">
         <v>125</v>
       </c>
-      <c r="E13" s="33" t="s">
+      <c r="E13" s="9" t="s">
         <v>126</v>
       </c>
-      <c r="F13" s="33" t="s">
+      <c r="F13" s="9" t="s">
         <v>91</v>
       </c>
-      <c r="G13" s="33" t="s">
+      <c r="G13" s="9" t="s">
         <v>108</v>
       </c>
-      <c r="H13" s="33" t="s">
+      <c r="H13" s="9" t="s">
         <v>109</v>
       </c>
-      <c r="I13" s="32" t="s">
+      <c r="I13" s="8" t="s">
         <v>127</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="62" customHeight="1">
-      <c r="A14" s="33" t="s">
+      <c r="A14" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="B14" s="33" t="s">
+      <c r="B14" s="9" t="s">
         <v>128</v>
       </c>
-      <c r="C14" s="33" t="s">
+      <c r="C14" s="9" t="s">
         <v>129</v>
       </c>
-      <c r="D14" s="33" t="s">
+      <c r="D14" s="9" t="s">
         <v>130</v>
       </c>
-      <c r="E14" s="33" t="s">
+      <c r="E14" s="9" t="s">
         <v>131</v>
       </c>
-      <c r="F14" s="33" t="s">
+      <c r="F14" s="9" t="s">
         <v>91</v>
       </c>
-      <c r="G14" s="33" t="s">
+      <c r="G14" s="9" t="s">
         <v>108</v>
       </c>
-      <c r="H14" s="33" t="s">
+      <c r="H14" s="9" t="s">
         <v>109</v>
       </c>
-      <c r="I14" s="32" t="s">
+      <c r="I14" s="8" t="s">
         <v>132</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="62" customHeight="1">
-      <c r="A15" s="33" t="s">
+      <c r="A15" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="B15" s="33" t="s">
+      <c r="B15" s="9" t="s">
         <v>133</v>
       </c>
-      <c r="C15" s="33" t="s">
+      <c r="C15" s="9" t="s">
         <v>134</v>
       </c>
-      <c r="D15" s="33" t="s">
+      <c r="D15" s="9" t="s">
         <v>125</v>
       </c>
-      <c r="E15" s="33" t="s">
+      <c r="E15" s="9" t="s">
         <v>126</v>
       </c>
-      <c r="F15" s="33" t="s">
+      <c r="F15" s="9" t="s">
         <v>91</v>
       </c>
-      <c r="G15" s="33" t="s">
+      <c r="G15" s="9" t="s">
         <v>108</v>
       </c>
-      <c r="H15" s="33" t="s">
+      <c r="H15" s="9" t="s">
         <v>109</v>
       </c>
-      <c r="I15" s="32" t="s">
+      <c r="I15" s="8" t="s">
         <v>132</v>
       </c>
     </row>
     <row r="16" spans="1:9" ht="62" customHeight="1">
-      <c r="A16" s="33" t="s">
+      <c r="A16" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="B16" s="33" t="s">
+      <c r="B16" s="9" t="s">
         <v>135</v>
       </c>
-      <c r="C16" s="33" t="s">
+      <c r="C16" s="9" t="s">
         <v>136</v>
       </c>
-      <c r="D16" s="33" t="s">
+      <c r="D16" s="9" t="s">
         <v>137</v>
       </c>
-      <c r="E16" s="33" t="s">
+      <c r="E16" s="9" t="s">
         <v>138</v>
       </c>
-      <c r="F16" s="33" t="s">
+      <c r="F16" s="9" t="s">
         <v>91</v>
       </c>
-      <c r="G16" s="33" t="s">
+      <c r="G16" s="9" t="s">
         <v>115</v>
       </c>
-      <c r="H16" s="33" t="s">
+      <c r="H16" s="9" t="s">
         <v>109</v>
       </c>
-      <c r="I16" s="32" t="s">
+      <c r="I16" s="8" t="s">
         <v>139</v>
       </c>
     </row>
     <row r="17" spans="1:9" ht="82" customHeight="1">
-      <c r="A17" s="34" t="s">
+      <c r="A17" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="B17" s="34" t="s">
+      <c r="B17" s="10" t="s">
         <v>140</v>
       </c>
-      <c r="C17" s="34" t="s">
+      <c r="C17" s="10" t="s">
         <v>141</v>
       </c>
-      <c r="D17" s="34" t="s">
+      <c r="D17" s="10" t="s">
         <v>142</v>
       </c>
-      <c r="E17" s="34" t="s">
+      <c r="E17" s="10" t="s">
         <v>143</v>
       </c>
-      <c r="F17" s="34" t="s">
+      <c r="F17" s="10" t="s">
         <v>91</v>
       </c>
-      <c r="G17" s="34" t="s">
+      <c r="G17" s="10" t="s">
         <v>144</v>
       </c>
-      <c r="H17" s="34" t="s">
+      <c r="H17" s="10" t="s">
         <v>109</v>
       </c>
       <c r="I17" s="7" t="s">
@@ -2193,28 +2302,28 @@
       </c>
     </row>
     <row r="18" spans="1:9" ht="82" customHeight="1">
-      <c r="A18" s="34" t="s">
+      <c r="A18" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="B18" s="34" t="s">
+      <c r="B18" s="10" t="s">
         <v>146</v>
       </c>
-      <c r="C18" s="34" t="s">
+      <c r="C18" s="10" t="s">
         <v>147</v>
       </c>
-      <c r="D18" s="34" t="s">
+      <c r="D18" s="10" t="s">
         <v>148</v>
       </c>
-      <c r="E18" s="34" t="s">
+      <c r="E18" s="10" t="s">
         <v>149</v>
       </c>
-      <c r="F18" s="34" t="s">
+      <c r="F18" s="10" t="s">
         <v>91</v>
       </c>
-      <c r="G18" s="34" t="s">
+      <c r="G18" s="10" t="s">
         <v>144</v>
       </c>
-      <c r="H18" s="34" t="s">
+      <c r="H18" s="10" t="s">
         <v>109</v>
       </c>
       <c r="I18" s="7" t="s">
@@ -2222,28 +2331,28 @@
       </c>
     </row>
     <row r="19" spans="1:9" ht="82" customHeight="1">
-      <c r="A19" s="34" t="s">
+      <c r="A19" s="10" t="s">
         <v>74</v>
       </c>
-      <c r="B19" s="34" t="s">
+      <c r="B19" s="10" t="s">
         <v>151</v>
       </c>
-      <c r="C19" s="34" t="s">
+      <c r="C19" s="10" t="s">
         <v>152</v>
       </c>
-      <c r="D19" s="34" t="s">
+      <c r="D19" s="10" t="s">
         <v>153</v>
       </c>
-      <c r="E19" s="34" t="s">
+      <c r="E19" s="10" t="s">
         <v>154</v>
       </c>
-      <c r="F19" s="34" t="s">
+      <c r="F19" s="10" t="s">
         <v>91</v>
       </c>
-      <c r="G19" s="34" t="s">
+      <c r="G19" s="10" t="s">
         <v>144</v>
       </c>
-      <c r="H19" s="34" t="s">
+      <c r="H19" s="10" t="s">
         <v>109</v>
       </c>
       <c r="I19" s="7" t="s">
@@ -2251,54 +2360,85 @@
       </c>
     </row>
     <row r="20" spans="1:9" ht="165" customHeight="1">
-      <c r="A20" s="34" t="s">
+      <c r="A20" s="10" t="s">
         <v>80</v>
       </c>
-      <c r="B20" s="34" t="s">
+      <c r="B20" s="10" t="s">
         <v>155</v>
       </c>
-      <c r="C20" s="34" t="s">
+      <c r="C20" s="10" t="s">
         <v>156</v>
       </c>
-      <c r="D20" s="34" t="s">
+      <c r="D20" s="10" t="s">
         <v>157</v>
       </c>
-      <c r="E20" s="34" t="s">
+      <c r="E20" s="10" t="s">
         <v>158</v>
       </c>
-      <c r="F20" s="34" t="s">
+      <c r="F20" s="10" t="s">
         <v>91</v>
       </c>
-      <c r="G20" s="34" t="s">
+      <c r="G20" s="10" t="s">
         <v>144</v>
       </c>
-      <c r="H20" s="34" t="s">
+      <c r="H20" s="10" t="s">
         <v>109</v>
       </c>
       <c r="I20" s="7" t="s">
         <v>159</v>
       </c>
     </row>
+    <row r="21" spans="1:9" ht="42">
+      <c r="A21" s="10" t="s">
+        <v>273</v>
+      </c>
+      <c r="B21" s="7" t="s">
+        <v>285</v>
+      </c>
+      <c r="C21" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="D21" s="7" t="s">
+        <v>282</v>
+      </c>
+      <c r="E21" s="7" t="s">
+        <v>279</v>
+      </c>
+      <c r="F21" s="10" t="s">
+        <v>92</v>
+      </c>
+      <c r="G21" s="10" t="s">
+        <v>284</v>
+      </c>
+      <c r="H21" s="10" t="s">
+        <v>109</v>
+      </c>
+      <c r="I21" s="37" t="s">
+        <v>283</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="C5:D5"/>
-    <mergeCell ref="E5:F5"/>
-    <mergeCell ref="G5:H5"/>
-    <mergeCell ref="A7:I7"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A2:I2"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="C4:D4"/>
     <mergeCell ref="E4:F4"/>
     <mergeCell ref="G4:H4"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="E5:F5"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="A7:I7"/>
   </mergeCells>
+  <phoneticPr fontId="14" type="noConversion"/>
   <dataValidations count="1">
     <dataValidation type="list" sqref="F9:F16" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"PASS,FAIL,BLOCKED,NOT RUN"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2320,55 +2460,55 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="32" customHeight="1">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="13" t="s">
         <v>160</v>
       </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
-      <c r="G1" s="8"/>
-      <c r="H1" s="8"/>
-      <c r="I1" s="8"/>
-      <c r="J1" s="8"/>
-      <c r="K1" s="8"/>
-      <c r="L1" s="8"/>
-      <c r="M1" s="8"/>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
+      <c r="H1" s="13"/>
+      <c r="I1" s="13"/>
+      <c r="J1" s="13"/>
+      <c r="K1" s="13"/>
+      <c r="L1" s="13"/>
+      <c r="M1" s="13"/>
     </row>
     <row r="2" spans="1:13" ht="30" customHeight="1">
-      <c r="A2" s="9" t="s">
+      <c r="A2" s="14" t="s">
         <v>161</v>
       </c>
-      <c r="B2" s="9"/>
-      <c r="C2" s="9"/>
-      <c r="D2" s="9"/>
-      <c r="E2" s="9"/>
-      <c r="F2" s="9"/>
-      <c r="G2" s="9"/>
-      <c r="H2" s="9"/>
-      <c r="I2" s="9"/>
-      <c r="J2" s="9"/>
-      <c r="K2" s="9"/>
-      <c r="L2" s="9"/>
-      <c r="M2" s="9"/>
+      <c r="B2" s="14"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="14"/>
+      <c r="G2" s="14"/>
+      <c r="H2" s="14"/>
+      <c r="I2" s="14"/>
+      <c r="J2" s="14"/>
+      <c r="K2" s="14"/>
+      <c r="L2" s="14"/>
+      <c r="M2" s="14"/>
     </row>
     <row r="4" spans="1:13" ht="30" customHeight="1">
-      <c r="A4" s="10" t="s">
+      <c r="A4" s="12" t="s">
         <v>162</v>
       </c>
-      <c r="B4" s="10"/>
-      <c r="C4" s="10"/>
-      <c r="D4" s="10"/>
-      <c r="E4" s="10"/>
-      <c r="F4" s="10"/>
-      <c r="G4" s="10"/>
-      <c r="H4" s="10"/>
-      <c r="I4" s="10"/>
-      <c r="J4" s="10"/>
-      <c r="K4" s="10"/>
-      <c r="L4" s="10"/>
-      <c r="M4" s="10"/>
+      <c r="B4" s="12"/>
+      <c r="C4" s="12"/>
+      <c r="D4" s="12"/>
+      <c r="E4" s="12"/>
+      <c r="F4" s="12"/>
+      <c r="G4" s="12"/>
+      <c r="H4" s="12"/>
+      <c r="I4" s="12"/>
+      <c r="J4" s="12"/>
+      <c r="K4" s="12"/>
+      <c r="L4" s="12"/>
+      <c r="M4" s="12"/>
     </row>
     <row r="5" spans="1:13" ht="34" customHeight="1">
       <c r="A5" s="1" t="s">
@@ -2412,37 +2552,37 @@
       </c>
     </row>
     <row r="6" spans="1:13" ht="85" customHeight="1">
-      <c r="A6" s="33" t="s">
+      <c r="A6" s="9" t="s">
         <v>171</v>
       </c>
-      <c r="B6" s="33" t="s">
+      <c r="B6" s="9" t="s">
         <v>172</v>
       </c>
-      <c r="C6" s="33" t="s">
+      <c r="C6" s="9" t="s">
         <v>173</v>
       </c>
-      <c r="D6" s="33" t="s">
+      <c r="D6" s="9" t="s">
         <v>174</v>
       </c>
-      <c r="E6" s="33" t="s">
+      <c r="E6" s="9" t="s">
         <v>175</v>
       </c>
-      <c r="F6" s="33" t="s">
+      <c r="F6" s="9" t="s">
         <v>176</v>
       </c>
-      <c r="G6" s="32" t="s">
+      <c r="G6" s="8" t="s">
         <v>177</v>
       </c>
-      <c r="H6" s="32" t="s">
+      <c r="H6" s="8" t="s">
         <v>178</v>
       </c>
-      <c r="I6" s="32" t="s">
+      <c r="I6" s="8" t="s">
         <v>179</v>
       </c>
-      <c r="J6" s="33" t="s">
+      <c r="J6" s="9" t="s">
         <v>180</v>
       </c>
-      <c r="K6" s="33" t="s">
+      <c r="K6" s="9" t="s">
         <v>181</v>
       </c>
       <c r="L6" s="2" t="s">
@@ -2453,37 +2593,37 @@
       </c>
     </row>
     <row r="7" spans="1:13" ht="85" customHeight="1">
-      <c r="A7" s="33" t="s">
+      <c r="A7" s="9" t="s">
         <v>183</v>
       </c>
-      <c r="B7" s="33" t="s">
+      <c r="B7" s="9" t="s">
         <v>184</v>
       </c>
-      <c r="C7" s="33" t="s">
+      <c r="C7" s="9" t="s">
         <v>185</v>
       </c>
-      <c r="D7" s="33" t="s">
+      <c r="D7" s="9" t="s">
         <v>174</v>
       </c>
-      <c r="E7" s="33" t="s">
+      <c r="E7" s="9" t="s">
         <v>186</v>
       </c>
-      <c r="F7" s="33" t="s">
+      <c r="F7" s="9" t="s">
         <v>187</v>
       </c>
-      <c r="G7" s="32" t="s">
+      <c r="G7" s="8" t="s">
         <v>188</v>
       </c>
-      <c r="H7" s="32" t="s">
+      <c r="H7" s="8" t="s">
         <v>189</v>
       </c>
-      <c r="I7" s="32" t="s">
+      <c r="I7" s="8" t="s">
         <v>190</v>
       </c>
-      <c r="J7" s="33" t="s">
+      <c r="J7" s="9" t="s">
         <v>191</v>
       </c>
-      <c r="K7" s="33" t="s">
+      <c r="K7" s="9" t="s">
         <v>181</v>
       </c>
       <c r="L7" s="2" t="s">
@@ -2494,37 +2634,37 @@
       </c>
     </row>
     <row r="8" spans="1:13" ht="85" customHeight="1">
-      <c r="A8" s="33" t="s">
+      <c r="A8" s="9" t="s">
         <v>192</v>
       </c>
-      <c r="B8" s="33" t="s">
+      <c r="B8" s="9" t="s">
         <v>193</v>
       </c>
-      <c r="C8" s="33" t="s">
+      <c r="C8" s="9" t="s">
         <v>194</v>
       </c>
-      <c r="D8" s="33" t="s">
+      <c r="D8" s="9" t="s">
         <v>174</v>
       </c>
-      <c r="E8" s="33" t="s">
+      <c r="E8" s="9" t="s">
         <v>195</v>
       </c>
-      <c r="F8" s="33" t="s">
+      <c r="F8" s="9" t="s">
         <v>196</v>
       </c>
-      <c r="G8" s="32" t="s">
+      <c r="G8" s="8" t="s">
         <v>197</v>
       </c>
-      <c r="H8" s="32" t="s">
+      <c r="H8" s="8" t="s">
         <v>198</v>
       </c>
-      <c r="I8" s="32" t="s">
+      <c r="I8" s="8" t="s">
         <v>199</v>
       </c>
-      <c r="J8" s="33" t="s">
+      <c r="J8" s="9" t="s">
         <v>200</v>
       </c>
-      <c r="K8" s="33" t="s">
+      <c r="K8" s="9" t="s">
         <v>201</v>
       </c>
       <c r="L8" s="2" t="s">
@@ -2535,37 +2675,37 @@
       </c>
     </row>
     <row r="9" spans="1:13" ht="85" customHeight="1">
-      <c r="A9" s="33" t="s">
+      <c r="A9" s="9" t="s">
         <v>202</v>
       </c>
-      <c r="B9" s="33" t="s">
+      <c r="B9" s="9" t="s">
         <v>203</v>
       </c>
-      <c r="C9" s="33" t="s">
+      <c r="C9" s="9" t="s">
         <v>173</v>
       </c>
-      <c r="D9" s="33" t="s">
+      <c r="D9" s="9" t="s">
         <v>174</v>
       </c>
-      <c r="E9" s="33" t="s">
+      <c r="E9" s="9" t="s">
         <v>204</v>
       </c>
-      <c r="F9" s="33" t="s">
+      <c r="F9" s="9" t="s">
         <v>187</v>
       </c>
-      <c r="G9" s="32" t="s">
+      <c r="G9" s="8" t="s">
         <v>205</v>
       </c>
-      <c r="H9" s="32" t="s">
+      <c r="H9" s="8" t="s">
         <v>206</v>
       </c>
-      <c r="I9" s="32" t="s">
+      <c r="I9" s="8" t="s">
         <v>207</v>
       </c>
-      <c r="J9" s="33" t="s">
+      <c r="J9" s="9" t="s">
         <v>200</v>
       </c>
-      <c r="K9" s="33" t="s">
+      <c r="K9" s="9" t="s">
         <v>201</v>
       </c>
       <c r="L9" s="2" t="s">
@@ -2576,37 +2716,37 @@
       </c>
     </row>
     <row r="10" spans="1:13" ht="85" customHeight="1">
-      <c r="A10" s="33" t="s">
+      <c r="A10" s="9" t="s">
         <v>208</v>
       </c>
-      <c r="B10" s="33" t="s">
+      <c r="B10" s="9" t="s">
         <v>209</v>
       </c>
-      <c r="C10" s="33" t="s">
+      <c r="C10" s="9" t="s">
         <v>210</v>
       </c>
-      <c r="D10" s="33" t="s">
+      <c r="D10" s="9" t="s">
         <v>211</v>
       </c>
-      <c r="E10" s="33" t="s">
+      <c r="E10" s="9" t="s">
         <v>212</v>
       </c>
-      <c r="F10" s="33" t="s">
+      <c r="F10" s="9" t="s">
         <v>213</v>
       </c>
-      <c r="G10" s="32" t="s">
+      <c r="G10" s="8" t="s">
         <v>214</v>
       </c>
-      <c r="H10" s="32" t="s">
+      <c r="H10" s="8" t="s">
         <v>215</v>
       </c>
-      <c r="I10" s="32" t="s">
+      <c r="I10" s="8" t="s">
         <v>216</v>
       </c>
-      <c r="J10" s="33" t="s">
+      <c r="J10" s="9" t="s">
         <v>200</v>
       </c>
-      <c r="K10" s="33" t="s">
+      <c r="K10" s="9" t="s">
         <v>201</v>
       </c>
       <c r="L10" s="2" t="s">
@@ -2617,37 +2757,37 @@
       </c>
     </row>
     <row r="11" spans="1:13" ht="85" customHeight="1">
-      <c r="A11" s="33" t="s">
+      <c r="A11" s="9" t="s">
         <v>217</v>
       </c>
-      <c r="B11" s="33" t="s">
+      <c r="B11" s="9" t="s">
         <v>193</v>
       </c>
-      <c r="C11" s="33" t="s">
+      <c r="C11" s="9" t="s">
         <v>194</v>
       </c>
-      <c r="D11" s="33" t="s">
+      <c r="D11" s="9" t="s">
         <v>218</v>
       </c>
-      <c r="E11" s="33" t="s">
+      <c r="E11" s="9" t="s">
         <v>219</v>
       </c>
-      <c r="F11" s="33" t="s">
+      <c r="F11" s="9" t="s">
         <v>220</v>
       </c>
-      <c r="G11" s="32" t="s">
+      <c r="G11" s="8" t="s">
         <v>197</v>
       </c>
-      <c r="H11" s="32" t="s">
+      <c r="H11" s="8" t="s">
         <v>221</v>
       </c>
-      <c r="I11" s="32" t="s">
+      <c r="I11" s="8" t="s">
         <v>222</v>
       </c>
-      <c r="J11" s="33" t="s">
+      <c r="J11" s="9" t="s">
         <v>200</v>
       </c>
-      <c r="K11" s="33" t="s">
+      <c r="K11" s="9" t="s">
         <v>201</v>
       </c>
       <c r="L11" s="2" t="s">
@@ -2658,37 +2798,37 @@
       </c>
     </row>
     <row r="12" spans="1:13" ht="85" customHeight="1">
-      <c r="A12" s="33" t="s">
+      <c r="A12" s="9" t="s">
         <v>223</v>
       </c>
-      <c r="B12" s="33" t="s">
+      <c r="B12" s="9" t="s">
         <v>224</v>
       </c>
-      <c r="C12" s="33" t="s">
+      <c r="C12" s="9" t="s">
         <v>173</v>
       </c>
-      <c r="D12" s="33" t="s">
+      <c r="D12" s="9" t="s">
         <v>225</v>
       </c>
-      <c r="E12" s="33" t="s">
+      <c r="E12" s="9" t="s">
         <v>226</v>
       </c>
-      <c r="F12" s="33" t="s">
+      <c r="F12" s="9" t="s">
         <v>227</v>
       </c>
-      <c r="G12" s="32" t="s">
+      <c r="G12" s="8" t="s">
         <v>228</v>
       </c>
-      <c r="H12" s="32" t="s">
+      <c r="H12" s="8" t="s">
         <v>229</v>
       </c>
-      <c r="I12" s="32" t="s">
+      <c r="I12" s="8" t="s">
         <v>230</v>
       </c>
-      <c r="J12" s="33" t="s">
+      <c r="J12" s="9" t="s">
         <v>200</v>
       </c>
-      <c r="K12" s="33" t="s">
+      <c r="K12" s="9" t="s">
         <v>231</v>
       </c>
       <c r="L12" s="2" t="s">
@@ -2718,7 +2858,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:H40"/>
+  <dimension ref="A1:H41"/>
   <sheetFormatPr defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -2727,28 +2867,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="30" customHeight="1">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="33" t="s">
         <v>232</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="16"/>
-      <c r="H1" s="16"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
+      <c r="G1" s="33"/>
+      <c r="H1" s="33"/>
     </row>
     <row r="2" spans="1:8" ht="34" customHeight="1">
-      <c r="A2" s="17" t="s">
+      <c r="A2" s="34" t="s">
         <v>233</v>
       </c>
-      <c r="B2" s="17"/>
-      <c r="C2" s="17"/>
-      <c r="D2" s="17"/>
-      <c r="E2" s="17"/>
-      <c r="F2" s="17"/>
-      <c r="G2" s="17"/>
-      <c r="H2" s="17"/>
+      <c r="B2" s="34"/>
+      <c r="C2" s="34"/>
+      <c r="D2" s="34"/>
+      <c r="E2" s="34"/>
+      <c r="F2" s="34"/>
+      <c r="G2" s="34"/>
+      <c r="H2" s="34"/>
     </row>
     <row r="3" spans="1:8">
       <c r="A3" s="5"/>
@@ -2761,100 +2901,100 @@
       <c r="H3" s="5"/>
     </row>
     <row r="4" spans="1:8" ht="22" customHeight="1">
-      <c r="A4" s="18" t="s">
+      <c r="A4" s="22" t="s">
         <v>234</v>
       </c>
-      <c r="B4" s="18"/>
-      <c r="C4" s="18"/>
-      <c r="D4" s="18"/>
-      <c r="E4" s="18"/>
-      <c r="F4" s="18"/>
-      <c r="G4" s="18"/>
-      <c r="H4" s="18"/>
+      <c r="B4" s="22"/>
+      <c r="C4" s="22"/>
+      <c r="D4" s="22"/>
+      <c r="E4" s="22"/>
+      <c r="F4" s="22"/>
+      <c r="G4" s="22"/>
+      <c r="H4" s="22"/>
     </row>
     <row r="5" spans="1:8" ht="28" customHeight="1">
-      <c r="A5" s="19" t="s">
+      <c r="A5" s="31" t="s">
         <v>235</v>
       </c>
-      <c r="B5" s="19"/>
-      <c r="C5" s="20" t="s">
+      <c r="B5" s="31"/>
+      <c r="C5" s="32" t="s">
         <v>236</v>
       </c>
-      <c r="D5" s="20"/>
-      <c r="E5" s="20"/>
-      <c r="F5" s="20"/>
-      <c r="G5" s="20"/>
-      <c r="H5" s="20"/>
+      <c r="D5" s="32"/>
+      <c r="E5" s="32"/>
+      <c r="F5" s="32"/>
+      <c r="G5" s="32"/>
+      <c r="H5" s="32"/>
     </row>
     <row r="6" spans="1:8" ht="28" customHeight="1">
-      <c r="A6" s="19" t="s">
+      <c r="A6" s="31" t="s">
         <v>237</v>
       </c>
-      <c r="B6" s="19"/>
-      <c r="C6" s="20" t="s">
+      <c r="B6" s="31"/>
+      <c r="C6" s="32" t="s">
         <v>238</v>
       </c>
-      <c r="D6" s="20"/>
-      <c r="E6" s="20"/>
-      <c r="F6" s="20"/>
-      <c r="G6" s="20"/>
-      <c r="H6" s="20"/>
+      <c r="D6" s="32"/>
+      <c r="E6" s="32"/>
+      <c r="F6" s="32"/>
+      <c r="G6" s="32"/>
+      <c r="H6" s="32"/>
     </row>
     <row r="7" spans="1:8" ht="28" customHeight="1">
-      <c r="A7" s="19" t="s">
+      <c r="A7" s="31" t="s">
         <v>239</v>
       </c>
-      <c r="B7" s="19"/>
-      <c r="C7" s="20" t="s">
+      <c r="B7" s="31"/>
+      <c r="C7" s="32" t="s">
         <v>240</v>
       </c>
-      <c r="D7" s="20"/>
-      <c r="E7" s="20"/>
-      <c r="F7" s="20"/>
-      <c r="G7" s="20"/>
-      <c r="H7" s="20"/>
+      <c r="D7" s="32"/>
+      <c r="E7" s="32"/>
+      <c r="F7" s="32"/>
+      <c r="G7" s="32"/>
+      <c r="H7" s="32"/>
     </row>
     <row r="8" spans="1:8" ht="28" customHeight="1">
-      <c r="A8" s="19" t="s">
+      <c r="A8" s="31" t="s">
         <v>241</v>
       </c>
-      <c r="B8" s="19"/>
-      <c r="C8" s="20" t="s">
+      <c r="B8" s="31"/>
+      <c r="C8" s="32" t="s">
+        <v>286</v>
+      </c>
+      <c r="D8" s="32"/>
+      <c r="E8" s="32"/>
+      <c r="F8" s="32"/>
+      <c r="G8" s="32"/>
+      <c r="H8" s="32"/>
+    </row>
+    <row r="9" spans="1:8" ht="28" customHeight="1">
+      <c r="A9" s="31" t="s">
         <v>242</v>
       </c>
-      <c r="D8" s="20"/>
-      <c r="E8" s="20"/>
-      <c r="F8" s="20"/>
-      <c r="G8" s="20"/>
-      <c r="H8" s="20"/>
-    </row>
-    <row r="9" spans="1:8" ht="28" customHeight="1">
-      <c r="A9" s="19" t="s">
+      <c r="B9" s="31"/>
+      <c r="C9" s="32" t="s">
         <v>243</v>
       </c>
-      <c r="B9" s="19"/>
-      <c r="C9" s="20" t="s">
+      <c r="D9" s="32"/>
+      <c r="E9" s="32"/>
+      <c r="F9" s="32"/>
+      <c r="G9" s="32"/>
+      <c r="H9" s="32"/>
+    </row>
+    <row r="10" spans="1:8" ht="28" customHeight="1">
+      <c r="A10" s="31" t="s">
         <v>244</v>
       </c>
-      <c r="D9" s="20"/>
-      <c r="E9" s="20"/>
-      <c r="F9" s="20"/>
-      <c r="G9" s="20"/>
-      <c r="H9" s="20"/>
-    </row>
-    <row r="10" spans="1:8" ht="28" customHeight="1">
-      <c r="A10" s="19" t="s">
+      <c r="B10" s="31"/>
+      <c r="C10" s="32" t="s">
         <v>245</v>
       </c>
-      <c r="B10" s="19"/>
-      <c r="C10" s="20" t="s">
-        <v>246</v>
-      </c>
-      <c r="D10" s="20"/>
-      <c r="E10" s="20"/>
-      <c r="F10" s="20"/>
-      <c r="G10" s="20"/>
-      <c r="H10" s="20"/>
+      <c r="D10" s="32"/>
+      <c r="E10" s="32"/>
+      <c r="F10" s="32"/>
+      <c r="G10" s="32"/>
+      <c r="H10" s="32"/>
     </row>
     <row r="11" spans="1:8">
       <c r="A11" s="5"/>
@@ -2867,66 +3007,66 @@
       <c r="H11" s="5"/>
     </row>
     <row r="12" spans="1:8" ht="22" customHeight="1">
-      <c r="A12" s="18" t="s">
+      <c r="A12" s="22" t="s">
+        <v>246</v>
+      </c>
+      <c r="B12" s="22"/>
+      <c r="C12" s="22"/>
+      <c r="D12" s="22"/>
+      <c r="E12" s="22"/>
+      <c r="F12" s="22"/>
+      <c r="G12" s="22"/>
+      <c r="H12" s="22"/>
+    </row>
+    <row r="13" spans="1:8">
+      <c r="A13" s="26" t="s">
+        <v>90</v>
+      </c>
+      <c r="B13" s="26"/>
+      <c r="C13" s="27" t="s">
         <v>247</v>
       </c>
-      <c r="B12" s="18"/>
-      <c r="C12" s="18"/>
-      <c r="D12" s="18"/>
-      <c r="E12" s="18"/>
-      <c r="F12" s="18"/>
-      <c r="G12" s="18"/>
-      <c r="H12" s="18"/>
-    </row>
-    <row r="13" spans="1:8">
-      <c r="A13" s="21" t="s">
-        <v>90</v>
-      </c>
-      <c r="B13" s="21"/>
-      <c r="C13" s="22" t="s">
+      <c r="D13" s="27"/>
+      <c r="E13" s="28" t="s">
         <v>248</v>
       </c>
-      <c r="D13" s="22"/>
-      <c r="E13" s="23" t="s">
-        <v>249</v>
-      </c>
-      <c r="F13" s="23"/>
-      <c r="G13" s="24" t="s">
+      <c r="F13" s="28"/>
+      <c r="G13" s="29" t="s">
         <v>93</v>
       </c>
-      <c r="H13" s="24"/>
+      <c r="H13" s="29"/>
     </row>
     <row r="14" spans="1:8">
-      <c r="A14" s="25">
-        <f>COUNTA(Test_Execution!$A$9:$A$20)</f>
+      <c r="A14" s="30">
+        <f>COUNTA(Test_Execution!$A$9:$A$21)</f>
+        <v>13</v>
+      </c>
+      <c r="B14" s="30"/>
+      <c r="C14" s="30">
+        <f>COUNTIF(Test_Execution!$F$9:$F$21,"PASS")</f>
         <v>12</v>
       </c>
-      <c r="B14" s="25"/>
-      <c r="C14" s="25">
-        <f>COUNTIF(Test_Execution!$F$9:$F$20,"PASS")</f>
-        <v>12</v>
-      </c>
-      <c r="D14" s="25"/>
-      <c r="E14" s="25">
-        <f>COUNTIF(Test_Execution!$F$9:$F$20,"FAIL")</f>
+      <c r="D14" s="30"/>
+      <c r="E14" s="30">
+        <f>COUNTIF(Test_Execution!$F$9:$F$21,"FAIL")</f>
+        <v>1</v>
+      </c>
+      <c r="F14" s="30"/>
+      <c r="G14" s="30">
+        <f>COUNTIF(Test_Execution!$F$9:$F$21,"BLOCKED")</f>
         <v>0</v>
       </c>
-      <c r="F14" s="25"/>
-      <c r="G14" s="25">
-        <f>COUNTIF(Test_Execution!$F$9:$F$20,"BLOCKED")</f>
-        <v>0</v>
-      </c>
-      <c r="H14" s="25"/>
+      <c r="H14" s="30"/>
     </row>
     <row r="15" spans="1:8">
-      <c r="A15" s="25"/>
-      <c r="B15" s="25"/>
-      <c r="C15" s="25"/>
-      <c r="D15" s="25"/>
-      <c r="E15" s="25"/>
-      <c r="F15" s="25"/>
-      <c r="G15" s="25"/>
-      <c r="H15" s="25"/>
+      <c r="A15" s="30"/>
+      <c r="B15" s="30"/>
+      <c r="C15" s="30"/>
+      <c r="D15" s="30"/>
+      <c r="E15" s="30"/>
+      <c r="F15" s="30"/>
+      <c r="G15" s="30"/>
+      <c r="H15" s="30"/>
     </row>
     <row r="16" spans="1:8">
       <c r="A16" s="5"/>
@@ -2939,353 +3079,378 @@
       <c r="H16" s="5"/>
     </row>
     <row r="17" spans="1:8" ht="22" customHeight="1">
-      <c r="A17" s="18" t="s">
-        <v>250</v>
-      </c>
-      <c r="B17" s="18"/>
-      <c r="C17" s="18"/>
-      <c r="D17" s="18"/>
-      <c r="E17" s="18"/>
-      <c r="F17" s="18"/>
-      <c r="G17" s="18"/>
-      <c r="H17" s="18"/>
+      <c r="A17" s="22" t="s">
+        <v>249</v>
+      </c>
+      <c r="B17" s="22"/>
+      <c r="C17" s="22"/>
+      <c r="D17" s="22"/>
+      <c r="E17" s="22"/>
+      <c r="F17" s="22"/>
+      <c r="G17" s="22"/>
+      <c r="H17" s="22"/>
     </row>
     <row r="18" spans="1:8">
       <c r="A18" s="6" t="s">
+        <v>250</v>
+      </c>
+      <c r="B18" s="6" t="s">
         <v>251</v>
       </c>
-      <c r="B18" s="6" t="s">
+      <c r="C18" s="6" t="s">
         <v>252</v>
       </c>
-      <c r="C18" s="6" t="s">
+      <c r="D18" s="6" t="s">
         <v>253</v>
       </c>
-      <c r="D18" s="6" t="s">
+      <c r="E18" s="6" t="s">
         <v>254</v>
       </c>
-      <c r="E18" s="6" t="s">
+      <c r="F18" s="24" t="s">
         <v>255</v>
       </c>
-      <c r="F18" s="26" t="s">
-        <v>256</v>
-      </c>
-      <c r="G18" s="26"/>
-      <c r="H18" s="26"/>
+      <c r="G18" s="24"/>
+      <c r="H18" s="24"/>
     </row>
     <row r="19" spans="1:8" ht="38" customHeight="1">
       <c r="A19" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="B19" s="34">
+      <c r="B19" s="10">
         <f>COUNTA(Test_Execution!$A$9:$A$16)</f>
         <v>8</v>
       </c>
-      <c r="C19" s="34">
+      <c r="C19" s="10">
         <f>COUNTIF(Test_Execution!$F$9:$F$16,"PASS")</f>
         <v>8</v>
       </c>
-      <c r="D19" s="34">
+      <c r="D19" s="10">
         <f>COUNTIF(Test_Execution!$F$9:$F$16,"FAIL")</f>
         <v>0</v>
       </c>
-      <c r="E19" s="34">
+      <c r="E19" s="10">
         <f>COUNTIF(Test_Execution!$F$9:$F$16,"BLOCKED")</f>
         <v>0</v>
       </c>
-      <c r="F19" s="27" t="s">
-        <v>257</v>
-      </c>
-      <c r="G19" s="27"/>
-      <c r="H19" s="27"/>
+      <c r="F19" s="25" t="s">
+        <v>256</v>
+      </c>
+      <c r="G19" s="25"/>
+      <c r="H19" s="25"/>
     </row>
     <row r="20" spans="1:8" ht="38" customHeight="1">
       <c r="A20" s="7" t="s">
-        <v>258</v>
-      </c>
-      <c r="B20" s="34">
+        <v>257</v>
+      </c>
+      <c r="B20" s="10">
         <f>COUNTA(Test_Execution!$A$17:$A$19)</f>
         <v>3</v>
       </c>
-      <c r="C20" s="34">
+      <c r="C20" s="10">
         <f>COUNTIF(Test_Execution!$F$17:$F$19,"PASS")</f>
         <v>3</v>
       </c>
-      <c r="D20" s="34">
+      <c r="D20" s="10">
         <f>COUNTIF(Test_Execution!$F$17:$F$19,"FAIL")</f>
         <v>0</v>
       </c>
-      <c r="E20" s="34">
+      <c r="E20" s="10">
         <f>COUNTIF(Test_Execution!$F$17:$F$19,"BLOCKED")</f>
         <v>0</v>
       </c>
-      <c r="F20" s="27" t="s">
-        <v>259</v>
-      </c>
-      <c r="G20" s="27"/>
-      <c r="H20" s="27"/>
+      <c r="F20" s="25" t="s">
+        <v>258</v>
+      </c>
+      <c r="G20" s="25"/>
+      <c r="H20" s="25"/>
     </row>
     <row r="21" spans="1:8" ht="38" customHeight="1">
       <c r="A21" s="7" t="s">
-        <v>260</v>
-      </c>
-      <c r="B21" s="34">
+        <v>259</v>
+      </c>
+      <c r="B21" s="10">
         <f>COUNTA(Test_Execution!$A$20:$A$20)</f>
         <v>1</v>
       </c>
-      <c r="C21" s="34">
+      <c r="C21" s="10">
         <f>COUNTIF(Test_Execution!$F$20:$F$20,"PASS")</f>
         <v>1</v>
       </c>
-      <c r="D21" s="34">
+      <c r="D21" s="10">
         <f>COUNTIF(Test_Execution!$F$20:$F$20,"FAIL")</f>
         <v>0</v>
       </c>
-      <c r="E21" s="34">
+      <c r="E21" s="10">
         <f>COUNTIF(Test_Execution!$F$20:$F$20,"BLOCKED")</f>
         <v>0</v>
       </c>
-      <c r="F21" s="27" t="s">
+      <c r="F21" s="25" t="s">
+        <v>260</v>
+      </c>
+      <c r="G21" s="25"/>
+      <c r="H21" s="25"/>
+    </row>
+    <row r="22" spans="1:8" ht="38" customHeight="1">
+      <c r="A22" s="35" t="s">
+        <v>287</v>
+      </c>
+      <c r="B22" s="10">
+        <f>COUNTA(Test_Execution!$A$21:$A$21)</f>
+        <v>1</v>
+      </c>
+      <c r="C22" s="10">
+        <f>COUNTIF(Test_Execution!$F$21:$F$21,"PASS")</f>
+        <v>0</v>
+      </c>
+      <c r="D22" s="10">
+        <f>COUNTIF(Test_Execution!$F$21:$F$21,"FAIL")</f>
+        <v>1</v>
+      </c>
+      <c r="E22" s="10">
+        <f>COUNTIF(Test_Execution!$F$21:$F$21,"BLOCKED")</f>
+        <v>0</v>
+      </c>
+      <c r="F22" s="38" t="s">
+        <v>288</v>
+      </c>
+      <c r="G22" s="38"/>
+      <c r="H22" s="38"/>
+    </row>
+    <row r="23" spans="1:8">
+      <c r="A23" s="5"/>
+      <c r="B23" s="5"/>
+      <c r="C23" s="5"/>
+      <c r="D23" s="5"/>
+      <c r="E23" s="5"/>
+      <c r="F23" s="5"/>
+      <c r="G23" s="5"/>
+      <c r="H23" s="5"/>
+    </row>
+    <row r="24" spans="1:8" ht="22" customHeight="1">
+      <c r="A24" s="22" t="s">
         <v>261</v>
       </c>
-      <c r="G21" s="27"/>
-      <c r="H21" s="27"/>
-    </row>
-    <row r="22" spans="1:8">
-      <c r="A22" s="5"/>
-      <c r="B22" s="5"/>
-      <c r="C22" s="5"/>
-      <c r="D22" s="5"/>
-      <c r="E22" s="5"/>
-      <c r="F22" s="5"/>
-      <c r="G22" s="5"/>
-      <c r="H22" s="5"/>
-    </row>
-    <row r="23" spans="1:8" ht="22" customHeight="1">
-      <c r="A23" s="18" t="s">
+      <c r="B24" s="22"/>
+      <c r="C24" s="22"/>
+      <c r="D24" s="22"/>
+      <c r="E24" s="22"/>
+      <c r="F24" s="22"/>
+      <c r="G24" s="22"/>
+      <c r="H24" s="22"/>
+    </row>
+    <row r="25" spans="1:8" ht="44" customHeight="1">
+      <c r="A25" s="20" t="s">
         <v>262</v>
       </c>
-      <c r="B23" s="18"/>
-      <c r="C23" s="18"/>
-      <c r="D23" s="18"/>
-      <c r="E23" s="18"/>
-      <c r="F23" s="18"/>
-      <c r="G23" s="18"/>
-      <c r="H23" s="18"/>
-    </row>
-    <row r="24" spans="1:8" ht="44" customHeight="1">
-      <c r="A24" s="28" t="s">
+      <c r="B25" s="20"/>
+      <c r="C25" s="20"/>
+      <c r="D25" s="20"/>
+      <c r="E25" s="20"/>
+      <c r="F25" s="20"/>
+      <c r="G25" s="20"/>
+      <c r="H25" s="20"/>
+    </row>
+    <row r="26" spans="1:8" ht="44" customHeight="1">
+      <c r="A26" s="21" t="s">
         <v>263</v>
       </c>
-      <c r="B24" s="28"/>
-      <c r="C24" s="28"/>
-      <c r="D24" s="28"/>
-      <c r="E24" s="28"/>
-      <c r="F24" s="28"/>
-      <c r="G24" s="28"/>
-      <c r="H24" s="28"/>
-    </row>
-    <row r="25" spans="1:8" ht="44" customHeight="1">
-      <c r="A25" s="29" t="s">
+      <c r="B26" s="21"/>
+      <c r="C26" s="21"/>
+      <c r="D26" s="21"/>
+      <c r="E26" s="21"/>
+      <c r="F26" s="21"/>
+      <c r="G26" s="21"/>
+      <c r="H26" s="21"/>
+    </row>
+    <row r="27" spans="1:8" ht="44" customHeight="1">
+      <c r="A27" s="20" t="s">
         <v>264</v>
       </c>
-      <c r="B25" s="29"/>
-      <c r="C25" s="29"/>
-      <c r="D25" s="29"/>
-      <c r="E25" s="29"/>
-      <c r="F25" s="29"/>
-      <c r="G25" s="29"/>
-      <c r="H25" s="29"/>
-    </row>
-    <row r="26" spans="1:8" ht="44" customHeight="1">
-      <c r="A26" s="28" t="s">
+      <c r="B27" s="20"/>
+      <c r="C27" s="20"/>
+      <c r="D27" s="20"/>
+      <c r="E27" s="20"/>
+      <c r="F27" s="20"/>
+      <c r="G27" s="20"/>
+      <c r="H27" s="20"/>
+    </row>
+    <row r="28" spans="1:8" ht="44" customHeight="1">
+      <c r="A28" s="21" t="s">
         <v>265</v>
       </c>
-      <c r="B26" s="28"/>
-      <c r="C26" s="28"/>
-      <c r="D26" s="28"/>
-      <c r="E26" s="28"/>
-      <c r="F26" s="28"/>
-      <c r="G26" s="28"/>
-      <c r="H26" s="28"/>
-    </row>
-    <row r="27" spans="1:8" ht="44" customHeight="1">
-      <c r="A27" s="29" t="s">
+      <c r="B28" s="21"/>
+      <c r="C28" s="21"/>
+      <c r="D28" s="21"/>
+      <c r="E28" s="21"/>
+      <c r="F28" s="21"/>
+      <c r="G28" s="21"/>
+      <c r="H28" s="21"/>
+    </row>
+    <row r="29" spans="1:8" ht="34" customHeight="1">
+      <c r="A29" s="20" t="s">
         <v>266</v>
       </c>
-      <c r="B27" s="29"/>
-      <c r="C27" s="29"/>
-      <c r="D27" s="29"/>
-      <c r="E27" s="29"/>
-      <c r="F27" s="29"/>
-      <c r="G27" s="29"/>
-      <c r="H27" s="29"/>
-    </row>
-    <row r="28" spans="1:8" ht="34" customHeight="1">
-      <c r="A28" s="28" t="s">
+      <c r="B29" s="20"/>
+      <c r="C29" s="20"/>
+      <c r="D29" s="20"/>
+      <c r="E29" s="20"/>
+      <c r="F29" s="20"/>
+      <c r="G29" s="20"/>
+      <c r="H29" s="20"/>
+    </row>
+    <row r="30" spans="1:8" ht="44" customHeight="1">
+      <c r="A30" s="21" t="s">
         <v>267</v>
       </c>
-      <c r="B28" s="28"/>
-      <c r="C28" s="28"/>
-      <c r="D28" s="28"/>
-      <c r="E28" s="28"/>
-      <c r="F28" s="28"/>
-      <c r="G28" s="28"/>
-      <c r="H28" s="28"/>
-    </row>
-    <row r="29" spans="1:8" ht="44" customHeight="1">
-      <c r="A29" s="29" t="s">
+      <c r="B30" s="21"/>
+      <c r="C30" s="21"/>
+      <c r="D30" s="21"/>
+      <c r="E30" s="21"/>
+      <c r="F30" s="21"/>
+      <c r="G30" s="21"/>
+      <c r="H30" s="21"/>
+    </row>
+    <row r="31" spans="1:8">
+      <c r="A31" s="5"/>
+      <c r="B31" s="5"/>
+      <c r="C31" s="5"/>
+      <c r="D31" s="5"/>
+      <c r="E31" s="5"/>
+      <c r="F31" s="5"/>
+      <c r="G31" s="5"/>
+      <c r="H31" s="5"/>
+    </row>
+    <row r="32" spans="1:8" ht="22" customHeight="1">
+      <c r="A32" s="22" t="s">
         <v>268</v>
       </c>
-      <c r="B29" s="29"/>
-      <c r="C29" s="29"/>
-      <c r="D29" s="29"/>
-      <c r="E29" s="29"/>
-      <c r="F29" s="29"/>
-      <c r="G29" s="29"/>
-      <c r="H29" s="29"/>
-    </row>
-    <row r="30" spans="1:8">
-      <c r="A30" s="5"/>
-      <c r="B30" s="5"/>
-      <c r="C30" s="5"/>
-      <c r="D30" s="5"/>
-      <c r="E30" s="5"/>
-      <c r="F30" s="5"/>
-      <c r="G30" s="5"/>
-      <c r="H30" s="5"/>
-    </row>
-    <row r="31" spans="1:8" ht="22" customHeight="1">
-      <c r="A31" s="18" t="s">
+      <c r="B32" s="22"/>
+      <c r="C32" s="22"/>
+      <c r="D32" s="22"/>
+      <c r="E32" s="22"/>
+      <c r="F32" s="22"/>
+      <c r="G32" s="22"/>
+      <c r="H32" s="22"/>
+    </row>
+    <row r="33" spans="1:8" ht="30" customHeight="1">
+      <c r="A33" s="23" t="s">
+        <v>289</v>
+      </c>
+      <c r="B33" s="23"/>
+      <c r="C33" s="23"/>
+      <c r="D33" s="23"/>
+      <c r="E33" s="23"/>
+      <c r="F33" s="23"/>
+      <c r="G33" s="23"/>
+      <c r="H33" s="23"/>
+    </row>
+    <row r="34" spans="1:8" ht="30" customHeight="1">
+      <c r="A34" s="23"/>
+      <c r="B34" s="23"/>
+      <c r="C34" s="23"/>
+      <c r="D34" s="23"/>
+      <c r="E34" s="23"/>
+      <c r="F34" s="23"/>
+      <c r="G34" s="23"/>
+      <c r="H34" s="23"/>
+    </row>
+    <row r="35" spans="1:8" ht="30" customHeight="1">
+      <c r="A35" s="23"/>
+      <c r="B35" s="23"/>
+      <c r="C35" s="23"/>
+      <c r="D35" s="23"/>
+      <c r="E35" s="23"/>
+      <c r="F35" s="23"/>
+      <c r="G35" s="23"/>
+      <c r="H35" s="23"/>
+    </row>
+    <row r="36" spans="1:8">
+      <c r="A36" s="5"/>
+      <c r="B36" s="5"/>
+      <c r="C36" s="5"/>
+      <c r="D36" s="5"/>
+      <c r="E36" s="5"/>
+      <c r="F36" s="5"/>
+      <c r="G36" s="5"/>
+      <c r="H36" s="5"/>
+    </row>
+    <row r="37" spans="1:8" ht="22" customHeight="1">
+      <c r="A37" s="22" t="s">
         <v>269</v>
       </c>
-      <c r="B31" s="18"/>
-      <c r="C31" s="18"/>
-      <c r="D31" s="18"/>
-      <c r="E31" s="18"/>
-      <c r="F31" s="18"/>
-      <c r="G31" s="18"/>
-      <c r="H31" s="18"/>
-    </row>
-    <row r="32" spans="1:8" ht="30" customHeight="1">
-      <c r="A32" s="30" t="s">
+      <c r="B37" s="22"/>
+      <c r="C37" s="22"/>
+      <c r="D37" s="22"/>
+      <c r="E37" s="22"/>
+      <c r="F37" s="22"/>
+      <c r="G37" s="22"/>
+      <c r="H37" s="22"/>
+    </row>
+    <row r="38" spans="1:8" ht="30" customHeight="1">
+      <c r="A38" s="19" t="s">
         <v>270</v>
       </c>
-      <c r="B32" s="30"/>
-      <c r="C32" s="30"/>
-      <c r="D32" s="30"/>
-      <c r="E32" s="30"/>
-      <c r="F32" s="30"/>
-      <c r="G32" s="30"/>
-      <c r="H32" s="30"/>
-    </row>
-    <row r="33" spans="1:8" ht="30" customHeight="1">
-      <c r="A33" s="30"/>
-      <c r="B33" s="30"/>
-      <c r="C33" s="30"/>
-      <c r="D33" s="30"/>
-      <c r="E33" s="30"/>
-      <c r="F33" s="30"/>
-      <c r="G33" s="30"/>
-      <c r="H33" s="30"/>
-    </row>
-    <row r="34" spans="1:8" ht="30" customHeight="1">
-      <c r="A34" s="30"/>
-      <c r="B34" s="30"/>
-      <c r="C34" s="30"/>
-      <c r="D34" s="30"/>
-      <c r="E34" s="30"/>
-      <c r="F34" s="30"/>
-      <c r="G34" s="30"/>
-      <c r="H34" s="30"/>
-    </row>
-    <row r="35" spans="1:8">
-      <c r="A35" s="5"/>
-      <c r="B35" s="5"/>
-      <c r="C35" s="5"/>
-      <c r="D35" s="5"/>
-      <c r="E35" s="5"/>
-      <c r="F35" s="5"/>
-      <c r="G35" s="5"/>
-      <c r="H35" s="5"/>
-    </row>
-    <row r="36" spans="1:8" ht="22" customHeight="1">
-      <c r="A36" s="18" t="s">
+      <c r="B38" s="19"/>
+      <c r="C38" s="19"/>
+      <c r="D38" s="19"/>
+      <c r="E38" s="19"/>
+      <c r="F38" s="19"/>
+      <c r="G38" s="19"/>
+      <c r="H38" s="19"/>
+    </row>
+    <row r="39" spans="1:8" ht="30" customHeight="1">
+      <c r="A39" s="19" t="s">
         <v>271</v>
       </c>
-      <c r="B36" s="18"/>
-      <c r="C36" s="18"/>
-      <c r="D36" s="18"/>
-      <c r="E36" s="18"/>
-      <c r="F36" s="18"/>
-      <c r="G36" s="18"/>
-      <c r="H36" s="18"/>
-    </row>
-    <row r="37" spans="1:8" ht="30" customHeight="1">
-      <c r="A37" s="31" t="s">
+      <c r="B39" s="19"/>
+      <c r="C39" s="19"/>
+      <c r="D39" s="19"/>
+      <c r="E39" s="19"/>
+      <c r="F39" s="19"/>
+      <c r="G39" s="19"/>
+      <c r="H39" s="19"/>
+    </row>
+    <row r="40" spans="1:8" ht="30" customHeight="1">
+      <c r="A40" s="19" t="s">
         <v>272</v>
       </c>
-      <c r="B37" s="31"/>
-      <c r="C37" s="31"/>
-      <c r="D37" s="31"/>
-      <c r="E37" s="31"/>
-      <c r="F37" s="31"/>
-      <c r="G37" s="31"/>
-      <c r="H37" s="31"/>
-    </row>
-    <row r="38" spans="1:8" ht="30" customHeight="1">
-      <c r="A38" s="31" t="s">
-        <v>273</v>
-      </c>
-      <c r="B38" s="31"/>
-      <c r="C38" s="31"/>
-      <c r="D38" s="31"/>
-      <c r="E38" s="31"/>
-      <c r="F38" s="31"/>
-      <c r="G38" s="31"/>
-      <c r="H38" s="31"/>
-    </row>
-    <row r="39" spans="1:8" ht="30" customHeight="1">
-      <c r="A39" s="31" t="s">
-        <v>274</v>
-      </c>
-      <c r="B39" s="31"/>
-      <c r="C39" s="31"/>
-      <c r="D39" s="31"/>
-      <c r="E39" s="31"/>
-      <c r="F39" s="31"/>
-      <c r="G39" s="31"/>
-      <c r="H39" s="31"/>
-    </row>
-    <row r="40" spans="1:8">
-      <c r="A40" s="5"/>
-      <c r="B40" s="5"/>
-      <c r="C40" s="5"/>
-      <c r="D40" s="5"/>
-      <c r="E40" s="5"/>
-      <c r="F40" s="5"/>
-      <c r="G40" s="5"/>
-      <c r="H40" s="5"/>
+      <c r="B40" s="19"/>
+      <c r="C40" s="19"/>
+      <c r="D40" s="19"/>
+      <c r="E40" s="19"/>
+      <c r="F40" s="19"/>
+      <c r="G40" s="19"/>
+      <c r="H40" s="19"/>
+    </row>
+    <row r="41" spans="1:8">
+      <c r="A41" s="5"/>
+      <c r="B41" s="5"/>
+      <c r="C41" s="5"/>
+      <c r="D41" s="5"/>
+      <c r="E41" s="5"/>
+      <c r="F41" s="5"/>
+      <c r="G41" s="5"/>
+      <c r="H41" s="5"/>
     </row>
   </sheetData>
-  <mergeCells count="42">
-    <mergeCell ref="A37:H37"/>
-    <mergeCell ref="A38:H38"/>
-    <mergeCell ref="A39:H39"/>
-    <mergeCell ref="A28:H28"/>
-    <mergeCell ref="A29:H29"/>
-    <mergeCell ref="A31:H31"/>
-    <mergeCell ref="A32:H34"/>
-    <mergeCell ref="A36:H36"/>
-    <mergeCell ref="A23:H23"/>
-    <mergeCell ref="A24:H24"/>
-    <mergeCell ref="A25:H25"/>
-    <mergeCell ref="A26:H26"/>
-    <mergeCell ref="A27:H27"/>
-    <mergeCell ref="A17:H17"/>
-    <mergeCell ref="F18:H18"/>
-    <mergeCell ref="F19:H19"/>
-    <mergeCell ref="F20:H20"/>
-    <mergeCell ref="F21:H21"/>
+  <mergeCells count="43">
+    <mergeCell ref="F22:H22"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A4:H4"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="C5:H5"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="C6:H6"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="C7:H7"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="C8:H8"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="C9:H9"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="C10:H10"/>
+    <mergeCell ref="A12:H12"/>
     <mergeCell ref="A13:B13"/>
     <mergeCell ref="C13:D13"/>
     <mergeCell ref="E13:F13"/>
@@ -3294,22 +3459,24 @@
     <mergeCell ref="C14:D15"/>
     <mergeCell ref="E14:F15"/>
     <mergeCell ref="G14:H15"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="C9:H9"/>
-    <mergeCell ref="A10:B10"/>
-    <mergeCell ref="C10:H10"/>
-    <mergeCell ref="A12:H12"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="C6:H6"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="C7:H7"/>
-    <mergeCell ref="A8:B8"/>
-    <mergeCell ref="C8:H8"/>
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A4:H4"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="C5:H5"/>
+    <mergeCell ref="A17:H17"/>
+    <mergeCell ref="F18:H18"/>
+    <mergeCell ref="F19:H19"/>
+    <mergeCell ref="F20:H20"/>
+    <mergeCell ref="F21:H21"/>
+    <mergeCell ref="A24:H24"/>
+    <mergeCell ref="A25:H25"/>
+    <mergeCell ref="A26:H26"/>
+    <mergeCell ref="A27:H27"/>
+    <mergeCell ref="A28:H28"/>
+    <mergeCell ref="A38:H38"/>
+    <mergeCell ref="A39:H39"/>
+    <mergeCell ref="A40:H40"/>
+    <mergeCell ref="A29:H29"/>
+    <mergeCell ref="A30:H30"/>
+    <mergeCell ref="A32:H32"/>
+    <mergeCell ref="A33:H35"/>
+    <mergeCell ref="A37:H37"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>